<commit_message>
Split HEC-8572 Test IT import into one row per step
Co-authored-by: AndreiLitovko <AndreiLitovko@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/тест-кейсы/test-case-8572-testit.xlsx
+++ b/тест-кейсы/test-case-8572-testit.xlsx
@@ -66,11 +66,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
-    <col min="2" max="2" width="55" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
     <col min="4" max="4" width="70" customWidth="1"/>
     <col min="5" max="5" width="70" customWidth="1"/>
-    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -105,7 +105,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="220" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">HEC-8572. Скрытие личных данных в регистрации проб микробиологии по правам «Бюджет» и «Внебюджет»</t>
@@ -130,33 +130,273 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Открыть учётные данные пользователя и найти оба права «Просмотр личных данных».
-Войти пользователем с обоими правами. Открыть гриды «Регистрация проб / Внебюджет» и «Регистрация проб / Бюджет».
-Открыть запись каждого типа заказчика во внебюджете и в бюджете.
-Выключить право только для внебюджета, перезайти и открыть грид внебюджета.
-Открыть эти же внебюджетные записи.
-Не меняя права, открыть бюджетный грид и бюджетные записи.
-Включить внебюджет, выключить только бюджет и повторить проверки грида и формы.
-Выключить оба права и перезайти.
-Включить оба права и перезайти.</t>
+          <t xml:space="preserve">Открыть учётные данные пользователя и найти оба права «Просмотр личных данных».</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Оба права есть в пунктах бюджета и внебюджета и по умолчанию включены.
-Наименование, адрес, объекты и адреса объектов читаются.
-На форме «Наименование организации» и «Адрес» читаются. В таблице «Объекты, адреса объектов» колонки «Объекты» и «Адреса объектов» читаются.
-У всех трёх типов заказчика наименование, адрес, объекты и адреса объектов не читаются. Номер, дата и статус строки читаются.
-На форме наименование и адрес не читаются. В таблице объектов обе колонки не читаются у всех трёх типов заказчика.
-Наименование, адрес, объекты и адреса объектов читаются.
-Бюджетные данные не читаются. Внебюджетные читаются.
-Данные скрыты в обоих журналах, на форме и в таблице объектов.
-Данные снова читаются в обоих журналах и на формах.</t>
+          <t xml:space="preserve">Оба права есть в пунктах бюджета и внебюджета и по умолчанию включены.</t>
         </is>
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Личные данные заказчика в регистрации проб микробиологии скрываются только при выключенном праве «Просмотр личных данных» соответствующего журнала. Бюджет и внебюджет работают независимо. По умолчанию данные читаются. Скрытие действует в гриде, на форме и в таблице объектов для сторонней организации, субъекта и физического лица.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Войти пользователем с обоими правами. Открыть гриды «Регистрация проб / Внебюджет» и «Регистрация проб / Бюджет».</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Наименование, адрес, объекты и адреса объектов читаются.</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Открыть запись каждого типа заказчика во внебюджете и в бюджете.</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На форме «Наименование организации» и «Адрес» читаются. В таблице «Объекты, адреса объектов» колонки «Объекты» и «Адреса объектов» читаются.</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выключить право только для внебюджета, перезайти и открыть грид внебюджета.</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">У всех трёх типов заказчика наименование, адрес, объекты и адреса объектов не читаются. Номер, дата и статус строки читаются.</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Открыть эти же внебюджетные записи.</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">На форме наименование и адрес не читаются. В таблице объектов обе колонки не читаются у всех трёх типов заказчика.</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Не меняя права, открыть бюджетный грид и бюджетные записи.</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Наименование, адрес, объекты и адреса объектов читаются.</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Включить внебюджет, выключить только бюджет и повторить проверки грида и формы.</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Бюджетные данные не читаются. Внебюджетные читаются.</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выключить оба права и перезайти.</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Данные скрыты в обоих журналах, на форме и в таблице объектов.</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Включить оба права и перезайти.</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Данные снова читаются в обоих журналах и на формах.</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>